<commit_message>
Update tracking spreadsheet with send dates and open rates for batches 1-3
第1弾 sent 7/31 (77.78% open), 第2弾 sent 8/6 (20% open), 第3弾 sent 8/26
(merged former 第4弾's 3 contacts in, since they were sent together as
the final 13-contact send).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BR7yJNdjxAihJmydzi8ULT
</commit_message>
<xml_diff>
--- a/outreach/配信管理.xlsx
+++ b/outreach/配信管理.xlsx
@@ -666,11 +666,23 @@
           <t>中野区｜検証: contact.htmlに入力フォーム有、メールも記載</t>
         </is>
       </c>
-      <c r="L2" s="3" t="inlineStr"/>
-      <c r="M2" s="3" t="inlineStr"/>
+      <c r="L2" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>7/10 (77.78%)</t>
+        </is>
+      </c>
       <c r="N2" s="3" t="inlineStr"/>
       <c r="O2" s="3" t="inlineStr"/>
-      <c r="P2" s="3" t="inlineStr"/>
+      <c r="P2" s="3" t="inlineStr">
+        <is>
+          <t>送信済み</t>
+        </is>
+      </c>
       <c r="Q2" s="3" t="inlineStr"/>
       <c r="R2" s="3" t="inlineStr"/>
     </row>
@@ -730,11 +742,23 @@
           <t>新宿区山吹町｜検証: pet-joli.com/contact/にフォーム有、メールはプライバシー欄に記載</t>
         </is>
       </c>
-      <c r="L3" s="3" t="inlineStr"/>
-      <c r="M3" s="3" t="inlineStr"/>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>7/10 (77.78%)</t>
+        </is>
+      </c>
       <c r="N3" s="3" t="inlineStr"/>
       <c r="O3" s="3" t="inlineStr"/>
-      <c r="P3" s="3" t="inlineStr"/>
+      <c r="P3" s="3" t="inlineStr">
+        <is>
+          <t>送信済み</t>
+        </is>
+      </c>
       <c r="Q3" s="3" t="inlineStr"/>
       <c r="R3" s="3" t="inlineStr"/>
     </row>
@@ -790,11 +814,23 @@
           <t>名古屋市名東区｜検証: /contact/にフォーム有(氏名/メール/内容+CAPTCHA)、メールもテキスト公開、電話052-771-5866</t>
         </is>
       </c>
-      <c r="L4" s="3" t="inlineStr"/>
-      <c r="M4" s="3" t="inlineStr"/>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>7/10 (77.78%)</t>
+        </is>
+      </c>
       <c r="N4" s="3" t="inlineStr"/>
       <c r="O4" s="3" t="inlineStr"/>
-      <c r="P4" s="3" t="inlineStr"/>
+      <c r="P4" s="3" t="inlineStr">
+        <is>
+          <t>送信済み</t>
+        </is>
+      </c>
       <c r="Q4" s="3" t="inlineStr"/>
       <c r="R4" s="3" t="inlineStr"/>
     </row>
@@ -850,11 +886,23 @@
           <t>京都市/京都駅近く｜検証: トップに入力フォーム有(氏名/メール/予約・問合せ内容)、外部予約システムも</t>
         </is>
       </c>
-      <c r="L5" s="3" t="inlineStr"/>
-      <c r="M5" s="3" t="inlineStr"/>
+      <c r="L5" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="M5" s="3" t="inlineStr">
+        <is>
+          <t>7/10 (77.78%)</t>
+        </is>
+      </c>
       <c r="N5" s="3" t="inlineStr"/>
       <c r="O5" s="3" t="inlineStr"/>
-      <c r="P5" s="3" t="inlineStr"/>
+      <c r="P5" s="3" t="inlineStr">
+        <is>
+          <t>送信済み</t>
+        </is>
+      </c>
       <c r="Q5" s="3" t="inlineStr"/>
       <c r="R5" s="3" t="inlineStr"/>
     </row>
@@ -910,11 +958,23 @@
           <t>神戸市｜検証: contact.htmlにメール掲載、フォーム有(定期確認の旨記載)、電話・LINEも</t>
         </is>
       </c>
-      <c r="L6" s="3" t="inlineStr"/>
-      <c r="M6" s="3" t="inlineStr"/>
+      <c r="L6" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="M6" s="3" t="inlineStr">
+        <is>
+          <t>7/10 (77.78%)</t>
+        </is>
+      </c>
       <c r="N6" s="3" t="inlineStr"/>
       <c r="O6" s="3" t="inlineStr"/>
-      <c r="P6" s="3" t="inlineStr"/>
+      <c r="P6" s="3" t="inlineStr">
+        <is>
+          <t>送信済み</t>
+        </is>
+      </c>
       <c r="Q6" s="3" t="inlineStr"/>
       <c r="R6" s="3" t="inlineStr"/>
     </row>
@@ -970,11 +1030,23 @@
           <t>神戸市垂水区｜検証: /contact/にフォーム有(氏名/メール/電話/住所/ペット種別/メニュー/内容)、トップにもメール掲載</t>
         </is>
       </c>
-      <c r="L7" s="3" t="inlineStr"/>
-      <c r="M7" s="3" t="inlineStr"/>
+      <c r="L7" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="M7" s="3" t="inlineStr">
+        <is>
+          <t>7/10 (77.78%)</t>
+        </is>
+      </c>
       <c r="N7" s="3" t="inlineStr"/>
       <c r="O7" s="3" t="inlineStr"/>
-      <c r="P7" s="3" t="inlineStr"/>
+      <c r="P7" s="3" t="inlineStr">
+        <is>
+          <t>送信済み</t>
+        </is>
+      </c>
       <c r="Q7" s="3" t="inlineStr"/>
       <c r="R7" s="3" t="inlineStr"/>
     </row>
@@ -1030,11 +1102,23 @@
           <t>青森市本町｜フッターにmailto公開、/contact/に入力フォーム</t>
         </is>
       </c>
-      <c r="L8" s="3" t="inlineStr"/>
-      <c r="M8" s="3" t="inlineStr"/>
+      <c r="L8" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="M8" s="3" t="inlineStr">
+        <is>
+          <t>7/10 (77.78%)</t>
+        </is>
+      </c>
       <c r="N8" s="3" t="inlineStr"/>
       <c r="O8" s="3" t="inlineStr"/>
-      <c r="P8" s="3" t="inlineStr"/>
+      <c r="P8" s="3" t="inlineStr">
+        <is>
+          <t>送信済み</t>
+        </is>
+      </c>
       <c r="Q8" s="3" t="inlineStr"/>
       <c r="R8" s="3" t="inlineStr"/>
     </row>
@@ -1090,11 +1174,23 @@
           <t>三春町(田村郡)｜mailto公開、/contact/に入力フォーム</t>
         </is>
       </c>
-      <c r="L9" s="3" t="inlineStr"/>
-      <c r="M9" s="3" t="inlineStr"/>
+      <c r="L9" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="M9" s="3" t="inlineStr">
+        <is>
+          <t>7/10 (77.78%)</t>
+        </is>
+      </c>
       <c r="N9" s="3" t="inlineStr"/>
       <c r="O9" s="3" t="inlineStr"/>
-      <c r="P9" s="3" t="inlineStr"/>
+      <c r="P9" s="3" t="inlineStr">
+        <is>
+          <t>送信済み</t>
+        </is>
+      </c>
       <c r="Q9" s="3" t="inlineStr"/>
       <c r="R9" s="3" t="inlineStr"/>
     </row>
@@ -1150,11 +1246,23 @@
           <t>甲府市下石田｜フッターにメール公開、お問い合わせページに入力フォーム</t>
         </is>
       </c>
-      <c r="L10" s="3" t="inlineStr"/>
-      <c r="M10" s="3" t="inlineStr"/>
+      <c r="L10" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="M10" s="3" t="inlineStr">
+        <is>
+          <t>7/10 (77.78%)</t>
+        </is>
+      </c>
       <c r="N10" s="3" t="inlineStr"/>
       <c r="O10" s="3" t="inlineStr"/>
-      <c r="P10" s="3" t="inlineStr"/>
+      <c r="P10" s="3" t="inlineStr">
+        <is>
+          <t>送信済み</t>
+        </is>
+      </c>
       <c r="Q10" s="3" t="inlineStr"/>
       <c r="R10" s="3" t="inlineStr"/>
     </row>
@@ -1210,11 +1318,23 @@
           <t>三条市・長岡市｜トップにメール記載、/contactにフォームへのリンク</t>
         </is>
       </c>
-      <c r="L11" s="3" t="inlineStr"/>
-      <c r="M11" s="3" t="inlineStr"/>
+      <c r="L11" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="M11" s="3" t="inlineStr">
+        <is>
+          <t>7/10 (77.78%)</t>
+        </is>
+      </c>
       <c r="N11" s="3" t="inlineStr"/>
       <c r="O11" s="3" t="inlineStr"/>
-      <c r="P11" s="3" t="inlineStr"/>
+      <c r="P11" s="3" t="inlineStr">
+        <is>
+          <t>送信済み</t>
+        </is>
+      </c>
       <c r="Q11" s="3" t="inlineStr"/>
       <c r="R11" s="3" t="inlineStr"/>
     </row>
@@ -1270,11 +1390,23 @@
           <t>京都市北区紫野｜フッターにメール、/enquiry問い合わせ・/booking予約フォーム</t>
         </is>
       </c>
-      <c r="L12" s="3" t="inlineStr"/>
-      <c r="M12" s="3" t="inlineStr"/>
+      <c r="L12" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="M12" s="3" t="inlineStr">
+        <is>
+          <t>2/10 (20%)</t>
+        </is>
+      </c>
       <c r="N12" s="3" t="inlineStr"/>
       <c r="O12" s="3" t="inlineStr"/>
-      <c r="P12" s="3" t="inlineStr"/>
+      <c r="P12" s="3" t="inlineStr">
+        <is>
+          <t>送信済み</t>
+        </is>
+      </c>
       <c r="Q12" s="3" t="inlineStr"/>
       <c r="R12" s="3" t="inlineStr"/>
     </row>
@@ -1330,11 +1462,23 @@
           <t>山口市小郡光が丘｜フッターにmailto公開、/cms/pageask0.htmlに入力フォーム</t>
         </is>
       </c>
-      <c r="L13" s="3" t="inlineStr"/>
-      <c r="M13" s="3" t="inlineStr"/>
+      <c r="L13" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="M13" s="3" t="inlineStr">
+        <is>
+          <t>2/10 (20%)</t>
+        </is>
+      </c>
       <c r="N13" s="3" t="inlineStr"/>
       <c r="O13" s="3" t="inlineStr"/>
-      <c r="P13" s="3" t="inlineStr"/>
+      <c r="P13" s="3" t="inlineStr">
+        <is>
+          <t>送信済み</t>
+        </is>
+      </c>
       <c r="Q13" s="3" t="inlineStr"/>
       <c r="R13" s="3" t="inlineStr"/>
     </row>
@@ -1390,11 +1534,23 @@
           <t>徳島市八万町｜トップにメール公開、お問い合わせフォームリンク(予約は外部)</t>
         </is>
       </c>
-      <c r="L14" s="3" t="inlineStr"/>
-      <c r="M14" s="3" t="inlineStr"/>
+      <c r="L14" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="M14" s="3" t="inlineStr">
+        <is>
+          <t>2/10 (20%)</t>
+        </is>
+      </c>
       <c r="N14" s="3" t="inlineStr"/>
       <c r="O14" s="3" t="inlineStr"/>
-      <c r="P14" s="3" t="inlineStr"/>
+      <c r="P14" s="3" t="inlineStr">
+        <is>
+          <t>送信済み</t>
+        </is>
+      </c>
       <c r="Q14" s="3" t="inlineStr"/>
       <c r="R14" s="3" t="inlineStr"/>
     </row>
@@ -1450,11 +1606,23 @@
           <t>高知市仁井田｜/contactに入力フォーム、メールはプライバシーポリシー欄に記載</t>
         </is>
       </c>
-      <c r="L15" s="3" t="inlineStr"/>
-      <c r="M15" s="3" t="inlineStr"/>
+      <c r="L15" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="M15" s="3" t="inlineStr">
+        <is>
+          <t>2/10 (20%)</t>
+        </is>
+      </c>
       <c r="N15" s="3" t="inlineStr"/>
       <c r="O15" s="3" t="inlineStr"/>
-      <c r="P15" s="3" t="inlineStr"/>
+      <c r="P15" s="3" t="inlineStr">
+        <is>
+          <t>送信済み</t>
+        </is>
+      </c>
       <c r="Q15" s="3" t="inlineStr"/>
       <c r="R15" s="3" t="inlineStr"/>
     </row>
@@ -1510,11 +1678,23 @@
           <t>宮崎市(宮崎空港近く)｜会社情報欄にメール掲載、/nyawp/toiawase/に問い合わせフォーム</t>
         </is>
       </c>
-      <c r="L16" s="3" t="inlineStr"/>
-      <c r="M16" s="3" t="inlineStr"/>
+      <c r="L16" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="M16" s="3" t="inlineStr">
+        <is>
+          <t>2/10 (20%)</t>
+        </is>
+      </c>
       <c r="N16" s="3" t="inlineStr"/>
       <c r="O16" s="3" t="inlineStr"/>
-      <c r="P16" s="3" t="inlineStr"/>
+      <c r="P16" s="3" t="inlineStr">
+        <is>
+          <t>送信済み</t>
+        </is>
+      </c>
       <c r="Q16" s="3" t="inlineStr"/>
       <c r="R16" s="3" t="inlineStr"/>
     </row>
@@ -1570,11 +1750,23 @@
           <t>盛岡市菜園1丁目1-4｜フッターmailto公開、/contactに業者向けフォーム(一般予約はLINE/電話)</t>
         </is>
       </c>
-      <c r="L17" s="3" t="inlineStr"/>
-      <c r="M17" s="3" t="inlineStr"/>
+      <c r="L17" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="M17" s="3" t="inlineStr">
+        <is>
+          <t>2/10 (20%)</t>
+        </is>
+      </c>
       <c r="N17" s="3" t="inlineStr"/>
       <c r="O17" s="3" t="inlineStr"/>
-      <c r="P17" s="3" t="inlineStr"/>
+      <c r="P17" s="3" t="inlineStr">
+        <is>
+          <t>送信済み</t>
+        </is>
+      </c>
       <c r="Q17" s="3" t="inlineStr"/>
       <c r="R17" s="3" t="inlineStr"/>
     </row>
@@ -1630,11 +1822,23 @@
           <t>会津若松市行仁町7-22｜トップにメール、/contactに名前/メール/電話/内容の入力フォーム</t>
         </is>
       </c>
-      <c r="L18" s="3" t="inlineStr"/>
-      <c r="M18" s="3" t="inlineStr"/>
+      <c r="L18" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="M18" s="3" t="inlineStr">
+        <is>
+          <t>2/10 (20%)</t>
+        </is>
+      </c>
       <c r="N18" s="3" t="inlineStr"/>
       <c r="O18" s="3" t="inlineStr"/>
-      <c r="P18" s="3" t="inlineStr"/>
+      <c r="P18" s="3" t="inlineStr">
+        <is>
+          <t>送信済み</t>
+        </is>
+      </c>
       <c r="Q18" s="3" t="inlineStr"/>
       <c r="R18" s="3" t="inlineStr"/>
     </row>
@@ -1690,11 +1894,23 @@
           <t>富山市堀川本郷15-157｜/blank-3にフォーム+メール記載、予約は外部カレンダー</t>
         </is>
       </c>
-      <c r="L19" s="3" t="inlineStr"/>
-      <c r="M19" s="3" t="inlineStr"/>
+      <c r="L19" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="M19" s="3" t="inlineStr">
+        <is>
+          <t>2/10 (20%)</t>
+        </is>
+      </c>
       <c r="N19" s="3" t="inlineStr"/>
       <c r="O19" s="3" t="inlineStr"/>
-      <c r="P19" s="3" t="inlineStr"/>
+      <c r="P19" s="3" t="inlineStr">
+        <is>
+          <t>送信済み</t>
+        </is>
+      </c>
       <c r="Q19" s="3" t="inlineStr"/>
       <c r="R19" s="3" t="inlineStr"/>
     </row>
@@ -1750,11 +1966,23 @@
           <t>広島市南区上東雲町9-25｜/contact/にフォーム(CAPTCHA)+mailto掲載、別途予約システム</t>
         </is>
       </c>
-      <c r="L20" s="3" t="inlineStr"/>
-      <c r="M20" s="3" t="inlineStr"/>
+      <c r="L20" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="M20" s="3" t="inlineStr">
+        <is>
+          <t>2/10 (20%)</t>
+        </is>
+      </c>
       <c r="N20" s="3" t="inlineStr"/>
       <c r="O20" s="3" t="inlineStr"/>
-      <c r="P20" s="3" t="inlineStr"/>
+      <c r="P20" s="3" t="inlineStr">
+        <is>
+          <t>送信済み</t>
+        </is>
+      </c>
       <c r="Q20" s="3" t="inlineStr"/>
       <c r="R20" s="3" t="inlineStr"/>
     </row>
@@ -1810,11 +2038,23 @@
           <t>高知市春野町弘岡下2655-7｜フッターにメール掲載、/inquery/に名前/メール/題名/本文の入力フォーム</t>
         </is>
       </c>
-      <c r="L21" s="3" t="inlineStr"/>
-      <c r="M21" s="3" t="inlineStr"/>
+      <c r="L21" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="M21" s="3" t="inlineStr">
+        <is>
+          <t>2/10 (20%)</t>
+        </is>
+      </c>
       <c r="N21" s="3" t="inlineStr"/>
       <c r="O21" s="3" t="inlineStr"/>
-      <c r="P21" s="3" t="inlineStr"/>
+      <c r="P21" s="3" t="inlineStr">
+        <is>
+          <t>送信済み</t>
+        </is>
+      </c>
       <c r="Q21" s="3" t="inlineStr"/>
       <c r="R21" s="3" t="inlineStr"/>
     </row>
@@ -1866,11 +2106,23 @@
           <t>札幌市中央区｜検証: mailtoでメール公開、対応は電話/LINE/メール、入力フォームは無し</t>
         </is>
       </c>
-      <c r="L22" s="3" t="inlineStr"/>
-      <c r="M22" s="3" t="inlineStr"/>
+      <c r="L22" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="M22" s="3" t="inlineStr">
+        <is>
+          <t>1/13 (7.69%・集計中)</t>
+        </is>
+      </c>
       <c r="N22" s="3" t="inlineStr"/>
       <c r="O22" s="3" t="inlineStr"/>
-      <c r="P22" s="3" t="inlineStr"/>
+      <c r="P22" s="3" t="inlineStr">
+        <is>
+          <t>送信済み</t>
+        </is>
+      </c>
       <c r="Q22" s="3" t="inlineStr"/>
       <c r="R22" s="3" t="inlineStr"/>
     </row>
@@ -1922,11 +2174,23 @@
           <t>茅野市｜検証: mailtoリンク有、入力フォームは無し、電話0266-55-7135</t>
         </is>
       </c>
-      <c r="L23" s="3" t="inlineStr"/>
-      <c r="M23" s="3" t="inlineStr"/>
+      <c r="L23" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="M23" s="3" t="inlineStr">
+        <is>
+          <t>1/13 (7.69%・集計中)</t>
+        </is>
+      </c>
       <c r="N23" s="3" t="inlineStr"/>
       <c r="O23" s="3" t="inlineStr"/>
-      <c r="P23" s="3" t="inlineStr"/>
+      <c r="P23" s="3" t="inlineStr">
+        <is>
+          <t>送信済み</t>
+        </is>
+      </c>
       <c r="Q23" s="3" t="inlineStr"/>
       <c r="R23" s="3" t="inlineStr"/>
     </row>
@@ -1982,11 +2246,23 @@
           <t>堺市堺区｜検証: contactページにメール公開、入力フォームは無くメール送信案内、電話072-238-2666</t>
         </is>
       </c>
-      <c r="L24" s="3" t="inlineStr"/>
-      <c r="M24" s="3" t="inlineStr"/>
+      <c r="L24" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="M24" s="3" t="inlineStr">
+        <is>
+          <t>1/13 (7.69%・集計中)</t>
+        </is>
+      </c>
       <c r="N24" s="3" t="inlineStr"/>
       <c r="O24" s="3" t="inlineStr"/>
-      <c r="P24" s="3" t="inlineStr"/>
+      <c r="P24" s="3" t="inlineStr">
+        <is>
+          <t>送信済み</t>
+        </is>
+      </c>
       <c r="Q24" s="3" t="inlineStr"/>
       <c r="R24" s="3" t="inlineStr"/>
     </row>
@@ -2038,11 +2314,23 @@
           <t>熊本市東区｜検証: infomationページにメール記載、入力フォームは無く電話/メール/予約制</t>
         </is>
       </c>
-      <c r="L25" s="3" t="inlineStr"/>
-      <c r="M25" s="3" t="inlineStr"/>
+      <c r="L25" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="M25" s="3" t="inlineStr">
+        <is>
+          <t>1/13 (7.69%・集計中)</t>
+        </is>
+      </c>
       <c r="N25" s="3" t="inlineStr"/>
       <c r="O25" s="3" t="inlineStr"/>
-      <c r="P25" s="3" t="inlineStr"/>
+      <c r="P25" s="3" t="inlineStr">
+        <is>
+          <t>送信済み</t>
+        </is>
+      </c>
       <c r="Q25" s="3" t="inlineStr"/>
       <c r="R25" s="3" t="inlineStr"/>
     </row>
@@ -2094,11 +2382,23 @@
           <t>山辺町｜メール公開、予約は外部システム(petlife.asia)</t>
         </is>
       </c>
-      <c r="L26" s="3" t="inlineStr"/>
-      <c r="M26" s="3" t="inlineStr"/>
+      <c r="L26" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="M26" s="3" t="inlineStr">
+        <is>
+          <t>1/13 (7.69%・集計中)</t>
+        </is>
+      </c>
       <c r="N26" s="3" t="inlineStr"/>
       <c r="O26" s="3" t="inlineStr"/>
-      <c r="P26" s="3" t="inlineStr"/>
+      <c r="P26" s="3" t="inlineStr">
+        <is>
+          <t>送信済み</t>
+        </is>
+      </c>
       <c r="Q26" s="3" t="inlineStr"/>
       <c r="R26" s="3" t="inlineStr"/>
     </row>
@@ -2150,11 +2450,23 @@
           <t>名古屋市緑区・守山区｜/contactにアドレスをアット表記で公開、フォームはスパム対策で停止中</t>
         </is>
       </c>
-      <c r="L27" s="3" t="inlineStr"/>
-      <c r="M27" s="3" t="inlineStr"/>
+      <c r="L27" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="M27" s="3" t="inlineStr">
+        <is>
+          <t>1/13 (7.69%・集計中)</t>
+        </is>
+      </c>
       <c r="N27" s="3" t="inlineStr"/>
       <c r="O27" s="3" t="inlineStr"/>
-      <c r="P27" s="3" t="inlineStr"/>
+      <c r="P27" s="3" t="inlineStr">
+        <is>
+          <t>送信済み</t>
+        </is>
+      </c>
       <c r="Q27" s="3" t="inlineStr"/>
       <c r="R27" s="3" t="inlineStr"/>
     </row>
@@ -2206,11 +2518,23 @@
           <t>別府市石垣西｜問い合わせ用メール掲載(24時間受付)、Webフォームなし</t>
         </is>
       </c>
-      <c r="L28" s="3" t="inlineStr"/>
-      <c r="M28" s="3" t="inlineStr"/>
+      <c r="L28" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="M28" s="3" t="inlineStr">
+        <is>
+          <t>1/13 (7.69%・集計中)</t>
+        </is>
+      </c>
       <c r="N28" s="3" t="inlineStr"/>
       <c r="O28" s="3" t="inlineStr"/>
-      <c r="P28" s="3" t="inlineStr"/>
+      <c r="P28" s="3" t="inlineStr">
+        <is>
+          <t>送信済み</t>
+        </is>
+      </c>
       <c r="Q28" s="3" t="inlineStr"/>
       <c r="R28" s="3" t="inlineStr"/>
     </row>
@@ -2262,11 +2586,23 @@
           <t>盛岡市三ツ割1丁目9-8｜フッターにメール公開、予約は電話(019-656-1332)誘導</t>
         </is>
       </c>
-      <c r="L29" s="3" t="inlineStr"/>
-      <c r="M29" s="3" t="inlineStr"/>
+      <c r="L29" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="M29" s="3" t="inlineStr">
+        <is>
+          <t>1/13 (7.69%・集計中)</t>
+        </is>
+      </c>
       <c r="N29" s="3" t="inlineStr"/>
       <c r="O29" s="3" t="inlineStr"/>
-      <c r="P29" s="3" t="inlineStr"/>
+      <c r="P29" s="3" t="inlineStr">
+        <is>
+          <t>送信済み</t>
+        </is>
+      </c>
       <c r="Q29" s="3" t="inlineStr"/>
       <c r="R29" s="3" t="inlineStr"/>
     </row>
@@ -2318,11 +2654,23 @@
           <t>福島市陣場町6-14｜ACCESSにメール公開、予約はLINE中心で入力フォームなし</t>
         </is>
       </c>
-      <c r="L30" s="3" t="inlineStr"/>
-      <c r="M30" s="3" t="inlineStr"/>
+      <c r="L30" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="M30" s="3" t="inlineStr">
+        <is>
+          <t>1/13 (7.69%・集計中)</t>
+        </is>
+      </c>
       <c r="N30" s="3" t="inlineStr"/>
       <c r="O30" s="3" t="inlineStr"/>
-      <c r="P30" s="3" t="inlineStr"/>
+      <c r="P30" s="3" t="inlineStr">
+        <is>
+          <t>送信済み</t>
+        </is>
+      </c>
       <c r="Q30" s="3" t="inlineStr"/>
       <c r="R30" s="3" t="inlineStr"/>
     </row>
@@ -2374,18 +2722,30 @@
           <t>立川市(西立川駅徒歩2分)｜媒体向けメール記載、/contact404、予約は電話042-526-3925</t>
         </is>
       </c>
-      <c r="L31" s="3" t="inlineStr"/>
-      <c r="M31" s="3" t="inlineStr"/>
+      <c r="L31" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="M31" s="3" t="inlineStr">
+        <is>
+          <t>1/13 (7.69%・集計中)</t>
+        </is>
+      </c>
       <c r="N31" s="3" t="inlineStr"/>
       <c r="O31" s="3" t="inlineStr"/>
-      <c r="P31" s="3" t="inlineStr"/>
+      <c r="P31" s="3" t="inlineStr">
+        <is>
+          <t>送信済み</t>
+        </is>
+      </c>
       <c r="Q31" s="3" t="inlineStr"/>
       <c r="R31" s="3" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>第4弾</t>
+          <t>第3弾</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
@@ -2430,18 +2790,34 @@
           <t>つくば市学園の森3-29-6｜mailto公開、完全予約制でWEB予約は外部(bg3.power-k.jp)、入力フォームなし</t>
         </is>
       </c>
-      <c r="L32" s="3" t="inlineStr"/>
-      <c r="M32" s="3" t="inlineStr"/>
+      <c r="L32" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="M32" s="3" t="inlineStr">
+        <is>
+          <t>1/13 (7.69%・集計中)</t>
+        </is>
+      </c>
       <c r="N32" s="3" t="inlineStr"/>
       <c r="O32" s="3" t="inlineStr"/>
-      <c r="P32" s="3" t="inlineStr"/>
+      <c r="P32" s="3" t="inlineStr">
+        <is>
+          <t>送信済み</t>
+        </is>
+      </c>
       <c r="Q32" s="3" t="inlineStr"/>
-      <c r="R32" s="3" t="inlineStr"/>
+      <c r="R32" s="3" t="inlineStr">
+        <is>
+          <t>第3弾(残り全部)としてbatch3と合算送信</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
         <is>
-          <t>第4弾</t>
+          <t>第3弾</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
@@ -2486,18 +2862,34 @@
           <t>豊橋市南大清水町富士見366-3｜トップにメール明記、電話0532-25-3220、入力フォームなし</t>
         </is>
       </c>
-      <c r="L33" s="3" t="inlineStr"/>
-      <c r="M33" s="3" t="inlineStr"/>
+      <c r="L33" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="M33" s="3" t="inlineStr">
+        <is>
+          <t>1/13 (7.69%・集計中)</t>
+        </is>
+      </c>
       <c r="N33" s="3" t="inlineStr"/>
       <c r="O33" s="3" t="inlineStr"/>
-      <c r="P33" s="3" t="inlineStr"/>
+      <c r="P33" s="3" t="inlineStr">
+        <is>
+          <t>送信済み</t>
+        </is>
+      </c>
       <c r="Q33" s="3" t="inlineStr"/>
-      <c r="R33" s="3" t="inlineStr"/>
+      <c r="R33" s="3" t="inlineStr">
+        <is>
+          <t>第3弾(残り全部)としてbatch3と合算送信</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
         <is>
-          <t>第4弾</t>
+          <t>第3弾</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
@@ -2542,13 +2934,29 @@
           <t>大阪市(九条店/玉造店)｜トップにメール2箇所記載、予約はLINE/電話で入力フォームなし</t>
         </is>
       </c>
-      <c r="L34" s="3" t="inlineStr"/>
-      <c r="M34" s="3" t="inlineStr"/>
+      <c r="L34" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="M34" s="3" t="inlineStr">
+        <is>
+          <t>1/13 (7.69%・集計中)</t>
+        </is>
+      </c>
       <c r="N34" s="3" t="inlineStr"/>
       <c r="O34" s="3" t="inlineStr"/>
-      <c r="P34" s="3" t="inlineStr"/>
+      <c r="P34" s="3" t="inlineStr">
+        <is>
+          <t>送信済み</t>
+        </is>
+      </c>
       <c r="Q34" s="3" t="inlineStr"/>
-      <c r="R34" s="3" t="inlineStr"/>
+      <c r="R34" s="3" t="inlineStr">
+        <is>
+          <t>第3弾(残り全部)としてbatch3と合算送信</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="8" t="inlineStr">

</xml_diff>